<commit_message>
fixed bug where dt wasn't being set
</commit_message>
<xml_diff>
--- a/Excel_files/momohara_neveu_2021_control.xlsx
+++ b/Excel_files/momohara_neveu_2021_control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\udickman\pySNNAP\Excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EABE534-99AE-4112-9025-25B9DA53AC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC25E08D-9377-47B3-9FC9-4A53AB02B583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="716" activeTab="6" xr2:uid="{F0735362-4961-42D4-9F52-DCA2C5A03203}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="716" xr2:uid="{F0735362-4961-42D4-9F52-DCA2C5A03203}"/>
   </bookViews>
   <sheets>
     <sheet name="Neu" sheetId="3" r:id="rId1"/>
@@ -10905,7 +10905,7 @@
       <c r="JN17" s="17"/>
       <c r="JO17" s="17"/>
       <c r="JP17" s="20"/>
-      <c r="JQ17" s="44">
+      <c r="JQ17" s="14">
         <v>0.35</v>
       </c>
       <c r="JR17" s="17">

</xml_diff>